<commit_message>
Resolve questionnaire conflict: E evidence via clarification, Q6 states
E's seeded clarification reply now attaches a valid ISO 9001 certificate
and an HP authorisation letter, so E fails the questionnaire before
clarification and passes after. Demo question 6 is reworded and both
states are recorded in ground_truth.json and checked by the generator.
The source of truth in the repo is now the master copy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/suppliers/A/Prakash_Quotation_PD-BLR-Q-2026-0412.xlsx
+++ b/seed/suppliers/A/Prakash_Quotation_PD-BLR-Q-2026-0412.xlsx
@@ -449,7 +449,7 @@
         <v>Print &amp; Power</v>
       </c>
       <c r="B7" s="1">
-        <v>2188840</v>
+        <v>2186590</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +465,7 @@
         <v>GRAND TOTAL</v>
       </c>
       <c r="B9" s="1">
-        <v>14746123</v>
+        <v>14743873</v>
       </c>
     </row>
     <row r="11">
@@ -1096,11 +1096,11 @@
         <v>5</v>
       </c>
       <c r="D9" s="1">
-        <v>45000</v>
+        <v>44550</v>
       </c>
       <c r="E9" s="1">
         <f>C9*D9</f>
-        <v>225000</v>
+        <v>222750</v>
       </c>
     </row>
     <row r="10">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="E12" s="1">
         <f>SUM(E8:E11)</f>
-        <v>1188200</v>
+        <v>1185950</v>
       </c>
     </row>
     <row r="14">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="E20" s="1">
         <f>E12+E18</f>
-        <v>2188840</v>
+        <v>2186590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
phase 2: extraction and normalisation
One structured-output model call per document (zod-validated, one retry),
deterministic normalisation in code with a logged ledger (FX, pack size,
GST-inclusive, bundle split), extraction flags, quote terms and code-decided
questionnaire answers. Code-derived conversions are Inferred. /eval scores
extraction against ground truth and shows cost per supplier and run plus
run-to-run variance. A's prices retuned for the Q6 story.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/suppliers/A/Prakash_Quotation_PD-BLR-Q-2026-0412.xlsx
+++ b/seed/suppliers/A/Prakash_Quotation_PD-BLR-Q-2026-0412.xlsx
@@ -433,7 +433,7 @@
         <v>Computing</v>
       </c>
       <c r="B5" s="1">
-        <v>8419000</v>
+        <v>8230800</v>
       </c>
     </row>
     <row r="6">
@@ -441,7 +441,7 @@
         <v>Peripherals &amp; Storage</v>
       </c>
       <c r="B6" s="1">
-        <v>2295300</v>
+        <v>2268500</v>
       </c>
     </row>
     <row r="7">
@@ -449,7 +449,7 @@
         <v>Print &amp; Power</v>
       </c>
       <c r="B7" s="1">
-        <v>2186590</v>
+        <v>2171870</v>
       </c>
     </row>
     <row r="8">
@@ -457,7 +457,7 @@
         <v>Networking</v>
       </c>
       <c r="B8" s="1">
-        <v>1842983</v>
+        <v>1779204</v>
       </c>
     </row>
     <row r="9">
@@ -465,7 +465,7 @@
         <v>GRAND TOTAL</v>
       </c>
       <c r="B9" s="1">
-        <v>14743873</v>
+        <v>14450374</v>
       </c>
     </row>
     <row r="11">
@@ -552,11 +552,11 @@
         <v>60</v>
       </c>
       <c r="D8" s="1">
-        <v>72650</v>
+        <v>72580</v>
       </c>
       <c r="E8" s="1">
         <f>C8*D8</f>
-        <v>4359000</v>
+        <v>4354800</v>
       </c>
       <c r="F8" t="str">
         <v>Bundle price: laptop + backpack</v>
@@ -586,7 +586,7 @@
       </c>
       <c r="E10" s="1">
         <f>SUM(E8:E9)</f>
-        <v>5472000</v>
+        <v>5467800</v>
       </c>
     </row>
     <row r="12">
@@ -605,11 +605,11 @@
         <v>40</v>
       </c>
       <c r="D13" s="1">
-        <v>54100</v>
+        <v>50450</v>
       </c>
       <c r="E13" s="1">
         <f>C13*D13</f>
-        <v>2164000</v>
+        <v>2018000</v>
       </c>
       <c r="F13" t="str">
         <v>SFF, lab use</v>
@@ -626,11 +626,11 @@
         <v>20</v>
       </c>
       <c r="D14" s="1">
-        <v>39150</v>
+        <v>37250</v>
       </c>
       <c r="E14" s="1">
         <f>C14*D14</f>
-        <v>783000</v>
+        <v>745000</v>
       </c>
     </row>
     <row r="15">
@@ -639,7 +639,7 @@
       </c>
       <c r="E15" s="1">
         <f>SUM(E13:E14)</f>
-        <v>2947000</v>
+        <v>2763000</v>
       </c>
     </row>
     <row r="17">
@@ -648,7 +648,7 @@
       </c>
       <c r="E17" s="1">
         <f>E10+E15</f>
-        <v>8419000</v>
+        <v>8230800</v>
       </c>
     </row>
   </sheetData>
@@ -786,11 +786,11 @@
         <v>10</v>
       </c>
       <c r="D13" s="1">
-        <v>1250</v>
+        <v>1180</v>
       </c>
       <c r="E13" s="1">
         <f>C13*D13</f>
-        <v>12500</v>
+        <v>11800</v>
       </c>
       <c r="F13" t="str">
         <v>Balance qty; 60 included in laptop bundle</v>
@@ -825,11 +825,11 @@
         <v>60</v>
       </c>
       <c r="D15" s="1">
-        <v>1160</v>
+        <v>1080</v>
       </c>
       <c r="E15" s="1">
         <f>C15*D15</f>
-        <v>69600</v>
+        <v>64800</v>
       </c>
     </row>
     <row r="16">
@@ -843,11 +843,11 @@
         <v>70</v>
       </c>
       <c r="D16" s="1">
-        <v>2270</v>
+        <v>2160</v>
       </c>
       <c r="E16" s="1">
         <f>C16*D16</f>
-        <v>158900</v>
+        <v>151200</v>
       </c>
     </row>
     <row r="17">
@@ -861,11 +861,11 @@
         <v>50</v>
       </c>
       <c r="D17" s="1">
-        <v>2550</v>
+        <v>2450</v>
       </c>
       <c r="E17" s="1">
         <f>C17*D17</f>
-        <v>127500</v>
+        <v>122500</v>
       </c>
     </row>
     <row r="18">
@@ -879,11 +879,11 @@
         <v>20</v>
       </c>
       <c r="D18" s="1">
-        <v>4550</v>
+        <v>4320</v>
       </c>
       <c r="E18" s="1">
         <f>C18*D18</f>
-        <v>91000</v>
+        <v>86400</v>
       </c>
     </row>
     <row r="19">
@@ -915,11 +915,11 @@
         <v>50</v>
       </c>
       <c r="D20" s="1">
-        <v>1550</v>
+        <v>1470</v>
       </c>
       <c r="E20" s="1">
         <f>C20*D20</f>
-        <v>77500</v>
+        <v>73500</v>
       </c>
     </row>
     <row r="21">
@@ -928,7 +928,7 @@
       </c>
       <c r="E21" s="1">
         <f>SUM(E13:E20)</f>
-        <v>1146100</v>
+        <v>1119300</v>
       </c>
     </row>
     <row r="23">
@@ -990,7 +990,7 @@
       </c>
       <c r="E28" s="1">
         <f>E10+E21+E26</f>
-        <v>2295300</v>
+        <v>2268500</v>
       </c>
     </row>
   </sheetData>
@@ -1135,11 +1135,11 @@
         <v>40</v>
       </c>
       <c r="D11" s="1">
-        <v>6630</v>
+        <v>6370</v>
       </c>
       <c r="E11" s="1">
         <f>C11*D11</f>
-        <v>265200</v>
+        <v>254800</v>
       </c>
     </row>
     <row r="12">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="E12" s="1">
         <f>SUM(E8:E11)</f>
-        <v>1185950</v>
+        <v>1175550</v>
       </c>
     </row>
     <row r="14">
@@ -1203,11 +1203,11 @@
         <v>60</v>
       </c>
       <c r="D17" s="1">
-        <v>954</v>
+        <v>882</v>
       </c>
       <c r="E17" s="1">
         <f>C17*D17</f>
-        <v>57240</v>
+        <v>52920</v>
       </c>
     </row>
     <row r="18">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="E18" s="1">
         <f>SUM(E15:E17)</f>
-        <v>1000640</v>
+        <v>996320</v>
       </c>
     </row>
     <row r="20">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="E20" s="1">
         <f>E12+E18</f>
-        <v>2186590</v>
+        <v>2171870</v>
       </c>
     </row>
   </sheetData>
@@ -1313,11 +1313,11 @@
         <v>8</v>
       </c>
       <c r="D8" s="1">
-        <v>79001</v>
+        <v>75166</v>
       </c>
       <c r="E8" s="1">
         <f>C8*D8</f>
-        <v>632008</v>
+        <v>601328</v>
       </c>
     </row>
     <row r="9">
@@ -1331,11 +1331,11 @@
         <v>20</v>
       </c>
       <c r="D9" s="1">
-        <v>4295.2</v>
+        <v>4047.4</v>
       </c>
       <c r="E9" s="1">
         <f>C9*D9</f>
-        <v>85904</v>
+        <v>80948</v>
       </c>
     </row>
     <row r="10">
@@ -1349,11 +1349,11 @@
         <v>25</v>
       </c>
       <c r="D10" s="1">
-        <v>16697</v>
+        <v>16166</v>
       </c>
       <c r="E10" s="1">
         <f>C10*D10</f>
-        <v>417425</v>
+        <v>404150</v>
       </c>
     </row>
     <row r="11">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="E11" s="1">
         <f>SUM(E8:E10)</f>
-        <v>1135337</v>
+        <v>1086426</v>
       </c>
     </row>
     <row r="13">
@@ -1416,11 +1416,11 @@
         <v>400</v>
       </c>
       <c r="D18" s="1">
-        <v>153.4</v>
+        <v>139.24</v>
       </c>
       <c r="E18" s="1">
         <f>C18*D18</f>
-        <v>61360</v>
+        <v>55696</v>
       </c>
     </row>
     <row r="19">
@@ -1434,11 +1434,11 @@
         <v>10</v>
       </c>
       <c r="D19" s="1">
-        <v>11434.2</v>
+        <v>10985.8</v>
       </c>
       <c r="E19" s="1">
         <f>C19*D19</f>
-        <v>114342</v>
+        <v>109858</v>
       </c>
       <c r="F19" t="str">
         <v>Per box</v>
@@ -1455,11 +1455,11 @@
         <v>8</v>
       </c>
       <c r="D20" s="1">
-        <v>14455</v>
+        <v>13865</v>
       </c>
       <c r="E20" s="1">
         <f>C20*D20</f>
-        <v>115640</v>
+        <v>110920</v>
       </c>
     </row>
     <row r="21">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="E21" s="1">
         <f>SUM(E18:E20)</f>
-        <v>291342</v>
+        <v>276474</v>
       </c>
     </row>
     <row r="23">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="E23" s="1">
         <f>E11+E15+E21</f>
-        <v>1842983</v>
+        <v>1779204</v>
       </c>
     </row>
     <row r="25">

</xml_diff>